<commit_message>
feat: add gpt-o1-preview and deepseek-code-v2.5 model evaluation for 2024-gaokao-ii
</commit_message>
<xml_diff>
--- a/eval/gaokao/2024_高考数学测评结果.xlsx
+++ b/eval/gaokao/2024_高考数学测评结果.xlsx
@@ -1,23 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10908"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/admin/PycharmProjects/llm_math_slover/eval/gaokao/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEE18C48-69F6-0643-8A63-61FDA2B3BA93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A0E9F18-EC8A-7241-AC98-4EF0F2E1D5AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11040" yWindow="500" windowWidth="25400" windowHeight="28300" activeTab="1" xr2:uid="{6EE47979-1F85-C943-A2B4-72199E8A51B4}"/>
+    <workbookView xWindow="-14300" yWindow="-28300" windowWidth="51200" windowHeight="28300" activeTab="5" xr2:uid="{6EE47979-1F85-C943-A2B4-72199E8A51B4}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="openai" sheetId="2" r:id="rId2"/>
-    <sheet name="claude" sheetId="3" r:id="rId3"/>
-    <sheet name="llm-math-solver" sheetId="4" r:id="rId4"/>
-    <sheet name="deepseek-v2" sheetId="5" r:id="rId5"/>
+    <sheet name="全国卷2-标准答案" sheetId="1" r:id="rId1"/>
+    <sheet name="openai_o1_preview" sheetId="6" r:id="rId2"/>
+    <sheet name="openai_gpt-4o" sheetId="2" r:id="rId3"/>
+    <sheet name="claude" sheetId="3" r:id="rId4"/>
+    <sheet name="llm-math-solver" sheetId="4" r:id="rId5"/>
+    <sheet name="deepseek-code-v2.5" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="96">
   <si>
     <t>题目序号</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -420,7 +421,106 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>\frac{2\sqrt{3}}{13}</t>
+    <t>\dfrac{\sqrt{2}}{2}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>\dfrac{1}{2}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BC</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ABD</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AD</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>30^\circ;2 + 3\sqrt{2} + \sqrt{6}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>y - (e - 2) = (e - 1)(x - 1);a &gt; 1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>\dfrac{2\sqrt{39}}{13}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ACD</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>24;128</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>24;121</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>\dfrac{1}{8}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>30^\circ;2 + 2 \sqrt{2} + \sqrt{6}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>\dfrac{8}{\sqrt{65}}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>x_2 = \dfrac{1 + 4\sqrt{7}}{3},\quad y_2 = -\dfrac{2}{3}(1 + \sqrt{7})</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>\\frac{2\\sqrt{2}}{3}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>63/67.525</t>
+  </si>
+  <si>
+    <r>
+      <t>0.686;乙</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13.5"/>
+        <color theme="1"/>
+        <rFont val="Menlo-Regular"/>
+      </rPr>
+      <t>;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13.5"/>
+        <color theme="1"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>乙</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>frac{1}{2}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>24;111</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2\\sqrt{15}/15</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -428,7 +528,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -461,6 +561,22 @@
       <name val=".AppleSystemUIFont"/>
       <charset val="136"/>
     </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="等线"/>
+      <family val="2"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="13.5"/>
+      <color theme="1"/>
+      <name val="Microsoft YaHei"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -479,21 +595,34 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="58" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="超链接" xfId="1" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1066,6 +1195,612 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34F63CB6-47B3-454D-B40F-BFD8D04B93AD}">
+  <dimension ref="A1:I21"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="3" max="3" width="55.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G2">
+        <v>5</v>
+      </c>
+      <c r="H2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3">
+        <v>5</v>
+      </c>
+      <c r="F3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3">
+        <v>5</v>
+      </c>
+      <c r="H3" t="s">
+        <v>4</v>
+      </c>
+      <c r="I3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E4">
+        <v>5</v>
+      </c>
+      <c r="F4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G4">
+        <v>5</v>
+      </c>
+      <c r="H4" t="s">
+        <v>75</v>
+      </c>
+      <c r="I4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
+      </c>
+      <c r="F5" t="s">
+        <v>3</v>
+      </c>
+      <c r="G5">
+        <v>5</v>
+      </c>
+      <c r="H5" t="s">
+        <v>3</v>
+      </c>
+      <c r="I5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G6">
+        <v>5</v>
+      </c>
+      <c r="H6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7">
+        <v>5</v>
+      </c>
+      <c r="F7">
+        <v>2</v>
+      </c>
+      <c r="G7">
+        <v>5</v>
+      </c>
+      <c r="H7">
+        <v>2</v>
+      </c>
+      <c r="I7">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>5</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>5</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>5</v>
+      </c>
+      <c r="C9" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" t="s">
+        <v>76</v>
+      </c>
+      <c r="E9">
+        <v>5</v>
+      </c>
+      <c r="F9" t="s">
+        <v>76</v>
+      </c>
+      <c r="G9">
+        <v>5</v>
+      </c>
+      <c r="H9" t="s">
+        <v>86</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>6</v>
+      </c>
+      <c r="C10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" t="s">
+        <v>77</v>
+      </c>
+      <c r="E10">
+        <v>6</v>
+      </c>
+      <c r="F10" t="s">
+        <v>77</v>
+      </c>
+      <c r="G10">
+        <v>6</v>
+      </c>
+      <c r="H10" t="s">
+        <v>77</v>
+      </c>
+      <c r="I10">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>6</v>
+      </c>
+      <c r="C11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" t="s">
+        <v>78</v>
+      </c>
+      <c r="E11">
+        <v>6</v>
+      </c>
+      <c r="F11" t="s">
+        <v>78</v>
+      </c>
+      <c r="G11">
+        <v>6</v>
+      </c>
+      <c r="H11" t="s">
+        <v>78</v>
+      </c>
+      <c r="I11">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>6</v>
+      </c>
+      <c r="C12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" t="s">
+        <v>79</v>
+      </c>
+      <c r="E12">
+        <v>6</v>
+      </c>
+      <c r="F12" t="s">
+        <v>79</v>
+      </c>
+      <c r="G12">
+        <v>6</v>
+      </c>
+      <c r="H12" t="s">
+        <v>79</v>
+      </c>
+      <c r="I12">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>5</v>
+      </c>
+      <c r="C13">
+        <v>95</v>
+      </c>
+      <c r="D13">
+        <v>95</v>
+      </c>
+      <c r="E13">
+        <v>5</v>
+      </c>
+      <c r="F13">
+        <v>95</v>
+      </c>
+      <c r="G13">
+        <v>5</v>
+      </c>
+      <c r="H13">
+        <v>95</v>
+      </c>
+      <c r="I13">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="18">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>5</v>
+      </c>
+      <c r="C14" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14">
+        <v>5</v>
+      </c>
+      <c r="F14" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14">
+        <v>5</v>
+      </c>
+      <c r="H14" t="s">
+        <v>12</v>
+      </c>
+      <c r="I14">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>5</v>
+      </c>
+      <c r="C15" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" t="s">
+        <v>10</v>
+      </c>
+      <c r="E15">
+        <v>5</v>
+      </c>
+      <c r="F15" t="s">
+        <v>85</v>
+      </c>
+      <c r="G15">
+        <v>2</v>
+      </c>
+      <c r="H15" t="s">
+        <v>10</v>
+      </c>
+      <c r="I15">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="18">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>13</v>
+      </c>
+      <c r="C16" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" t="s">
+        <v>80</v>
+      </c>
+      <c r="E16">
+        <v>13</v>
+      </c>
+      <c r="F16" t="s">
+        <v>80</v>
+      </c>
+      <c r="G16">
+        <v>13</v>
+      </c>
+      <c r="H16" t="s">
+        <v>87</v>
+      </c>
+      <c r="I16">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="18">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>15</v>
+      </c>
+      <c r="C17" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" t="s">
+        <v>81</v>
+      </c>
+      <c r="E17">
+        <v>15</v>
+      </c>
+      <c r="F17" t="s">
+        <v>69</v>
+      </c>
+      <c r="G17">
+        <v>15</v>
+      </c>
+      <c r="H17" t="s">
+        <v>69</v>
+      </c>
+      <c r="I17">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="18">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18">
+        <v>7</v>
+      </c>
+      <c r="C18" t="s">
+        <v>15</v>
+      </c>
+      <c r="D18" t="s">
+        <v>82</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18" t="s">
+        <v>76</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18" t="s">
+        <v>88</v>
+      </c>
+      <c r="I18">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="18">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19">
+        <v>17</v>
+      </c>
+      <c r="C19" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" t="s">
+        <v>16</v>
+      </c>
+      <c r="E19">
+        <v>17</v>
+      </c>
+      <c r="F19" t="s">
+        <v>16</v>
+      </c>
+      <c r="G19">
+        <v>17</v>
+      </c>
+      <c r="H19" t="s">
+        <v>16</v>
+      </c>
+      <c r="I19">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20">
+        <v>5</v>
+      </c>
+      <c r="C20" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20">
+        <v>5</v>
+      </c>
+      <c r="F20" t="s">
+        <v>11</v>
+      </c>
+      <c r="G20">
+        <v>5</v>
+      </c>
+      <c r="H20" t="s">
+        <v>89</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="E21">
+        <v>123</v>
+      </c>
+      <c r="G21">
+        <v>120</v>
+      </c>
+      <c r="I21">
+        <v>113</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3ECDAE15-B17A-FC48-8ECB-305D3DD418B3}">
   <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
@@ -1673,7 +2408,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4E59A4D-2408-384F-A94A-C9EBEDD795E8}">
   <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
@@ -2278,7 +3013,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A6EB1BB-B789-E24B-B677-2ECE2DA17105}">
   <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
@@ -2884,9 +3619,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E766331C-8DF8-1C43-A946-51F632B991F7}">
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="3" max="3" width="55.83203125" bestFit="1" customWidth="1"/>
@@ -2931,6 +3666,24 @@
       <c r="C2" t="s">
         <v>3</v>
       </c>
+      <c r="D2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G2">
+        <v>5</v>
+      </c>
+      <c r="H2" t="s">
+        <v>3</v>
+      </c>
+      <c r="I2">
+        <v>5</v>
+      </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3">
@@ -2942,8 +3695,26 @@
       <c r="C3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="4" spans="1:9">
+      <c r="D3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3">
+        <v>5</v>
+      </c>
+      <c r="F3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3">
+        <v>5</v>
+      </c>
+      <c r="H3" t="s">
+        <v>4</v>
+      </c>
+      <c r="I3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="17" customHeight="1">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2952,6 +3723,24 @@
       </c>
       <c r="C4" t="s">
         <v>4</v>
+      </c>
+      <c r="D4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4">
+        <v>5</v>
+      </c>
+      <c r="F4" t="s">
+        <v>4</v>
+      </c>
+      <c r="G4">
+        <v>5</v>
+      </c>
+      <c r="H4" t="s">
+        <v>4</v>
+      </c>
+      <c r="I4">
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -2964,8 +3753,26 @@
       <c r="C5" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:9">
+      <c r="D5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5" t="s">
+        <v>3</v>
+      </c>
+      <c r="G5">
+        <v>5</v>
+      </c>
+      <c r="H5" t="s">
+        <v>3</v>
+      </c>
+      <c r="I5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="17" customHeight="1">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2973,6 +3780,24 @@
         <v>5</v>
       </c>
       <c r="C6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G6">
+        <v>5</v>
+      </c>
+      <c r="H6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I6">
         <v>5</v>
       </c>
     </row>
@@ -2985,6 +3810,24 @@
       </c>
       <c r="C7" t="s">
         <v>6</v>
+      </c>
+      <c r="D7" t="s">
+        <v>4</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G7">
+        <v>5</v>
+      </c>
+      <c r="H7" t="s">
+        <v>3</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -2997,6 +3840,24 @@
       <c r="C8" t="s">
         <v>4</v>
       </c>
+      <c r="D8" t="s">
+        <v>4</v>
+      </c>
+      <c r="E8">
+        <v>5</v>
+      </c>
+      <c r="F8" t="s">
+        <v>3</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8" t="s">
+        <v>3</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9">
@@ -3008,6 +3869,24 @@
       <c r="C9" t="s">
         <v>3</v>
       </c>
+      <c r="D9" t="s">
+        <v>3</v>
+      </c>
+      <c r="E9">
+        <v>5</v>
+      </c>
+      <c r="F9" t="s">
+        <v>3</v>
+      </c>
+      <c r="G9">
+        <v>5</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="I9">
+        <v>5</v>
+      </c>
     </row>
     <row r="10" spans="1:9">
       <c r="A10">
@@ -3019,6 +3898,24 @@
       <c r="C10" t="s">
         <v>7</v>
       </c>
+      <c r="D10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10">
+        <v>6</v>
+      </c>
+      <c r="F10" t="s">
+        <v>7</v>
+      </c>
+      <c r="G10">
+        <v>6</v>
+      </c>
+      <c r="H10" t="s">
+        <v>7</v>
+      </c>
+      <c r="I10">
+        <v>6</v>
+      </c>
     </row>
     <row r="11" spans="1:9">
       <c r="A11">
@@ -3030,6 +3927,24 @@
       <c r="C11" t="s">
         <v>8</v>
       </c>
+      <c r="D11" t="s">
+        <v>83</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11" t="s">
+        <v>83</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11" t="s">
+        <v>83</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:9">
       <c r="A12">
@@ -3041,6 +3956,24 @@
       <c r="C12" t="s">
         <v>9</v>
       </c>
+      <c r="D12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12">
+        <v>6</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+      <c r="G12">
+        <v>6</v>
+      </c>
+      <c r="H12" t="s">
+        <v>9</v>
+      </c>
+      <c r="I12">
+        <v>6</v>
+      </c>
     </row>
     <row r="13" spans="1:9">
       <c r="A13">
@@ -3052,6 +3985,24 @@
       <c r="C13">
         <v>95</v>
       </c>
+      <c r="D13">
+        <v>95</v>
+      </c>
+      <c r="E13">
+        <v>5</v>
+      </c>
+      <c r="F13">
+        <v>95</v>
+      </c>
+      <c r="G13">
+        <v>5</v>
+      </c>
+      <c r="H13">
+        <v>95</v>
+      </c>
+      <c r="I13">
+        <v>5</v>
+      </c>
     </row>
     <row r="14" spans="1:9" ht="18">
       <c r="A14">
@@ -3063,6 +4014,24 @@
       <c r="C14" t="s">
         <v>12</v>
       </c>
+      <c r="D14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14">
+        <v>5</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14" t="s">
+        <v>12</v>
+      </c>
+      <c r="I14">
+        <v>5</v>
+      </c>
     </row>
     <row r="15" spans="1:9">
       <c r="A15">
@@ -3074,6 +4043,24 @@
       <c r="C15" t="s">
         <v>10</v>
       </c>
+      <c r="D15" t="s">
+        <v>84</v>
+      </c>
+      <c r="E15">
+        <v>2</v>
+      </c>
+      <c r="F15" t="s">
+        <v>10</v>
+      </c>
+      <c r="G15">
+        <v>5</v>
+      </c>
+      <c r="H15" t="s">
+        <v>94</v>
+      </c>
+      <c r="I15">
+        <v>2</v>
+      </c>
     </row>
     <row r="16" spans="1:9" ht="18">
       <c r="A16">
@@ -3085,8 +4072,26 @@
       <c r="C16" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" ht="18">
+      <c r="D16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E16">
+        <v>13</v>
+      </c>
+      <c r="F16" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16">
+        <v>13</v>
+      </c>
+      <c r="H16" t="s">
+        <v>13</v>
+      </c>
+      <c r="I16">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="18">
       <c r="A17">
         <v>16</v>
       </c>
@@ -3096,8 +4101,26 @@
       <c r="C17" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" ht="18">
+      <c r="D17" t="s">
+        <v>14</v>
+      </c>
+      <c r="E17">
+        <v>15</v>
+      </c>
+      <c r="F17" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17">
+        <v>15</v>
+      </c>
+      <c r="H17" t="s">
+        <v>14</v>
+      </c>
+      <c r="I17">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="18">
       <c r="A18">
         <v>17</v>
       </c>
@@ -3107,14 +4130,26 @@
       <c r="C18" t="s">
         <v>15</v>
       </c>
-      <c r="D18" t="s">
-        <v>75</v>
+      <c r="D18">
+        <v>1</v>
       </c>
       <c r="E18">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" ht="18">
+      <c r="F18" t="s">
+        <v>91</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="21">
       <c r="A19">
         <v>18</v>
       </c>
@@ -3124,8 +4159,26 @@
       <c r="C19" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="20" spans="1:5">
+      <c r="D19" t="s">
+        <v>16</v>
+      </c>
+      <c r="E19">
+        <v>17</v>
+      </c>
+      <c r="F19" t="s">
+        <v>92</v>
+      </c>
+      <c r="G19">
+        <v>5</v>
+      </c>
+      <c r="H19" t="s">
+        <v>92</v>
+      </c>
+      <c r="I19">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
       <c r="A20">
         <v>19</v>
       </c>
@@ -3135,9 +4188,41 @@
       <c r="C20" t="s">
         <v>11</v>
       </c>
+      <c r="D20" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20">
+        <v>5</v>
+      </c>
+      <c r="F20" t="s">
+        <v>11</v>
+      </c>
+      <c r="G20">
+        <v>5</v>
+      </c>
+      <c r="H20" t="s">
+        <v>11</v>
+      </c>
+      <c r="I20">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="E21">
+        <v>104</v>
+      </c>
+      <c r="G21">
+        <v>95</v>
+      </c>
+      <c r="I21">
+        <v>92</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="F14" r:id="rId1" xr:uid="{BC3589BA-5903-0F4E-BBE3-E76DFFF5EC34}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>